<commit_message>
docs: agrega la hoja Sprint 2 al backlog (#161)
</commit_message>
<xml_diff>
--- a/G3_Backlog.xlsx
+++ b/G3_Backlog.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Sprint 0" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Roadmap" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Sprint 1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sprint 2" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Módulos'!$A$1:$F$7</definedName>
@@ -16,6 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sprint 0'!$A$1:$H$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Roadmap'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sprint 1'!$A$1:$H$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sprint 2'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21466,4 +21468,437 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col width="11" customWidth="1" style="29" min="1" max="1"/>
+    <col width="40" customWidth="1" style="29" min="2" max="2"/>
+    <col width="52" customWidth="1" style="29" min="3" max="3"/>
+    <col width="12" customWidth="1" style="29" min="4" max="4"/>
+    <col width="22" customWidth="1" style="29" min="5" max="5"/>
+    <col width="30" customWidth="1" style="29" min="6" max="6"/>
+    <col width="8" customWidth="1" style="29" min="7" max="7"/>
+    <col width="13" customWidth="1" style="29" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="29">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Entregable</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Módulo</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Depende de</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1" s="29">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>S2-01</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Congelar el contrato de Comanda</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>Contrato de Comanda (campos, estados y operaciones crear, listar y cerrar) escrito en un documento, y un stub compartido para que M5 y M6 prueben sin esperar</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>Juan Ignacio Riquelme</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1" s="29">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>S2-02</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Confirmar con los docentes los supuestos y la fecha de entrega</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Lista de supuestos del equipo llevada a los docentes y fecha de entrega confirmada por escrito (R06 y R20)</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Franco Martín Soler</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="29">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>S2-03</t>
+        </is>
+      </c>
+      <c r="B4" s="26" t="inlineStr">
+        <is>
+          <t>Review del Sprint 2 y revisión de riesgos (28/10)</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="inlineStr">
+        <is>
+          <t>Cada módulo muestra su ABM, revisión cruzada entre módulos, riesgos R01 y R04 revisados e informe del Sprint 2 con burndown</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="F4" s="26" t="inlineStr">
+        <is>
+          <t>S2-M1 a S2-M6</t>
+        </is>
+      </c>
+      <c r="G4" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1" s="29">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>S2-M1</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Implementar las entidades base y el ABM de productos y carta (M1 Productos y Carta)</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Entidades de producto (plato, postre y bebida) y de sección de la carta con su ABM y listado: HU-M1-01 a HU-M1-13, con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Franco Martín Soler</t>
+        </is>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="29">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>S2-M2</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Implementar las entidades base y el ABM de menús (M2 Menús y Promociones)</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Entidades de menú ejecutivo y menú del día con su ABM: HU-M2-01 a HU-M2-06, con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>Joaquín Cardoso Díaz</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>S2-M1</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1" s="29">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>S2-M3</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Implementar las entidades base y el ABM del salón (M3 Salón y Mozos)</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Entidades de sector, mesa y mozo con su ABM y listado: HU-M3-01 a HU-M3-12, con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Giuliano Giannoncelli</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="29">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>S2-M4</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Implementar las entidades base y la comanda (M4 Atención al Público)</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Entidad de cliente con su ABM y listado (HU-M4-01 a HU-M4-03) y comanda con crear, listar y cerrar (HU-M4-04, HU-M4-07 y HU-M4-09), con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Juan Ignacio Riquelme</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>S2-01, S2-M1, S2-M3</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1" s="29">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>S2-M5</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Implementar la entidad base y el ABM de reservas (M5 Reservas)</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Entidad Reserva con crear, modificar y listar: HU-M5-01 a HU-M5-03, con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Federico Cabaña</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>S2-M3, S2-M4</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1" s="29">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>S2-M6</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Implementar las entidades base y el ABM de medios de pago (M6 Pagos)</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Entidad de medio de pago con su ABM y listado: HU-M6-04 a HU-M6-07, con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Héctor Sánchez</t>
+        </is>
+      </c>
+      <c r="F10" s="23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H10"/>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,En curso,Hecha"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: agrega el plan y el mensaje del Sprint 3 (S3-01)
- Corre las fechas del roadmap: el Sprint 2 se pasó un día, el Sprint 3
  va del 31/10 al 06/11 (G2), el Sprint 4 del 07/11 al 13/11 y el Cierre
  del 14/11 al 15/11.
- Agrega las tareas, el reparto de HU, el camino crítico y los criterios
  de cierre del Sprint 3, y la hoja «Sprint 3» del backlog.
- Actualiza la fecha del G2 en los riesgos.
- Reemplaza la estimación por Puntos de Función por su versión 2.
</commit_message>
<xml_diff>
--- a/G3_Backlog.xlsx
+++ b/G3_Backlog.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Módulos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Story Map" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Sprint 0" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Roadmap" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Sprint 1" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sprint 2" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léeme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Story Map" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 0" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint 3" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Módulos'!$A$1:$F$7</definedName>
@@ -18,6 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Roadmap'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sprint 1'!$A$1:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Sprint 2'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sprint 3'!$A$1:$H$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -15594,7 +15596,7 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>29/10 – 04/11</t>
+          <t>31/10 – 06/11</t>
         </is>
       </c>
       <c r="C5" s="27" t="inlineStr">
@@ -15609,7 +15611,7 @@
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
-          <t>G2 · 04/11</t>
+          <t>G2 · 06/11</t>
         </is>
       </c>
     </row>
@@ -15621,7 +15623,7 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>05/11 – 11/11</t>
+          <t>07/11 – 13/11</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
@@ -15648,12 +15650,12 @@
       </c>
       <c r="B7" s="27" t="inlineStr">
         <is>
-          <t>12/11 – 15/11</t>
+          <t>14/11 – 15/11</t>
         </is>
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>4 días</t>
+          <t>2 días</t>
         </is>
       </c>
       <c r="D7" s="27" t="inlineStr">
@@ -21567,7 +21569,7 @@
       </c>
       <c r="H2" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
@@ -21607,7 +21609,7 @@
       </c>
       <c r="H3" s="16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
@@ -21647,7 +21649,7 @@
       </c>
       <c r="H4" s="26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
@@ -21687,7 +21689,7 @@
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
@@ -21727,7 +21729,7 @@
       </c>
       <c r="H6" s="18" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
@@ -21767,7 +21769,7 @@
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecha</t>
         </is>
       </c>
     </row>
@@ -21807,7 +21809,7 @@
       </c>
       <c r="H8" s="21" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa al Sprint 3</t>
         </is>
       </c>
     </row>
@@ -21847,7 +21849,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa al Sprint 3</t>
         </is>
       </c>
     </row>
@@ -21887,7 +21889,7 @@
       </c>
       <c r="H10" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasa al Sprint 3</t>
         </is>
       </c>
     </row>
@@ -21895,10 +21897,362 @@
   <autoFilter ref="A1:H10"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pendiente,En curso,Hecha"</formula1>
+      <formula1>"Pendiente,En curso,Hecha,Pasa al Sprint 3"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" style="29" min="1" max="1"/>
+    <col width="40" customWidth="1" style="29" min="2" max="2"/>
+    <col width="52" customWidth="1" style="29" min="3" max="3"/>
+    <col width="12" customWidth="1" style="29" min="4" max="4"/>
+    <col width="22" customWidth="1" style="29" min="5" max="5"/>
+    <col width="30" customWidth="1" style="29" min="6" max="6"/>
+    <col width="8" customWidth="1" style="29" min="7" max="7"/>
+    <col width="13" customWidth="1" style="29" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="29">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Tarea</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Entregable</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Módulo</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Depende de</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1" s="29">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>S3-01</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Plan y mensaje del Sprint 3</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>Plan del Sprint 3 en SPRINT-0/Plan-de-trabajo-Sprint.md (tareas, reparto de HU, camino crítico y criterios de cierre), hoja «Sprint 3» del backlog, mensaje al equipo y cards del tablero</t>
+        </is>
+      </c>
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>Franco Martín Soler</t>
+        </is>
+      </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1" s="29">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>S3-M1</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>Implementar crear, marcar como entregado y cerrar la comanda (M4 Atención al Público)</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Comanda con crear (HU-M4-04), marcar un producto como entregado (HU-M4-08) y cerrar (HU-M4-09), con pruebas y pantallas. HU reasignadas de M4</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Franco Martín Soler</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>S3-M4 (cliente, PR #196)</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1" s="29">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>S3-M2</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Implementar las promociones (M2 Menús y Promociones)</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Promociones con crear, modificar y finalizar (HU-M2-07 a HU-M2-09), con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Joaquín Cardoso Díaz</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1" s="29">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>S3-M3</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Implementar modificar y reabrir la comanda y cobrar una factura adeudada (M4 Atención al Público y M6 Pagos)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Modificar y reabrir una comanda (HU-M4-05 y HU-M4-10) y cobrar una factura adeudada (HU-M6-02), con pruebas y pantallas. HU reasignadas de M4 y M6</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>M4 y M6</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Giuliano Giannoncelli</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>S3-M1 (crear y cerrar comanda), S3-M6 (factura)</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1" s="29">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>S3-M4</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Integrar el cliente e implementar listar y eliminar comandas (M4 Atención al Público)</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Cliente en develop (HU-M4-01 a HU-M4-03, PR #196) y comandas con listar (HU-M4-07) y eliminar (HU-M4-06), con pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>Juan Ignacio Riquelme</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>S3-M1 (crear comanda)</t>
+        </is>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1" s="29">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>S3-M5</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Integrar el ABM de reservas e implementar las cancelaciones y la comanda desde una reserva (M5 Reservas)</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>ABM de reservas en develop (HU-M5-01 a HU-M5-03), cancelación anticipada y por ausencia (HU-M5-04 y HU-M5-05) y comanda a partir de una reserva (HU-M5-06), con pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
+        <is>
+          <t>Federico Cabaña</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>S3-M4 (cliente), S3-M1 (crear comanda)</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="29">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>S3-M6</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>Implementar los medios de pago, la factura y el comprobante (M6 Pagos)</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
+        <is>
+          <t>Medios de pago con su ABM y listado (HU-M6-04 a HU-M6-07), factura de una comanda (HU-M6-01) y comprobante de pago (HU-M6-03), con migración, pruebas y pantallas</t>
+        </is>
+      </c>
+      <c r="D8" s="23" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="inlineStr">
+        <is>
+          <t>Héctor Sánchez</t>
+        </is>
+      </c>
+      <c r="F8" s="23" t="inlineStr">
+        <is>
+          <t>S3-M1 (cerrar comanda), S3-M3 (cobro)</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H8"/>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,En curso,Hecha"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>